<commit_message>
changing name in excel file
</commit_message>
<xml_diff>
--- a/names.xlsx
+++ b/names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pann\Documents\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59D8C7D-FFF6-444C-B55D-C97BAB30527D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC9E28E-C6A4-48BD-AA2A-25DC71453D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1428" yWindow="1140" windowWidth="19692" windowHeight="12540" xr2:uid="{6E0B6FA1-1E21-48EB-97C7-51C497158CFA}"/>
   </bookViews>
@@ -36,34 +36,343 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
   <si>
     <t>Name</t>
   </si>
   <si>
-    <t>Test5</t>
-  </si>
-  <si>
-    <t>Test6</t>
-  </si>
-  <si>
-    <t>Joshua</t>
-  </si>
-  <si>
-    <t>Daniel</t>
-  </si>
-  <si>
-    <t>Rewis</t>
-  </si>
-  <si>
-    <t>Aron</t>
+    <t>BACHELOR OF ARTS IN CHRISTIAN STUDIES</t>
+  </si>
+  <si>
+    <t>Chen, Jiale</t>
+  </si>
+  <si>
+    <t>Fanuel Frankie</t>
+  </si>
+  <si>
+    <t>Farman Rehmat</t>
+  </si>
+  <si>
+    <t>Gao, Wanli</t>
+  </si>
+  <si>
+    <t>Jerome Benggon</t>
+  </si>
+  <si>
+    <t>Jocelyn Abigail Olivier</t>
+  </si>
+  <si>
+    <t>Moo Wah</t>
+  </si>
+  <si>
+    <t>Saranyu Kamolprapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tum Sopheak Elijah </t>
+  </si>
+  <si>
+    <t>Sun, Huiyi</t>
+  </si>
+  <si>
+    <t>Surasak Tharapasook</t>
+  </si>
+  <si>
+    <t>Syaher Airil</t>
+  </si>
+  <si>
+    <t>Yang, Xun</t>
+  </si>
+  <si>
+    <t>Yu, Dawei</t>
+  </si>
+  <si>
+    <t>BACHELOR OF ARTS IN ENGLISH</t>
+  </si>
+  <si>
+    <t>Emphasis in English for Business</t>
+  </si>
+  <si>
+    <t>Mi Lian Za</t>
+  </si>
+  <si>
+    <t>Emphasis in English for Communication</t>
+  </si>
+  <si>
+    <t>Leandra Faith Remond</t>
+  </si>
+  <si>
+    <t>Olie Natalie Nelson</t>
+  </si>
+  <si>
+    <t>Sarah Ann Van Hee</t>
+  </si>
+  <si>
+    <t>Thet Darni Nyunt</t>
+  </si>
+  <si>
+    <t>Emphasis in Teaching English to Speakers of Other Languages (TESOL)</t>
+  </si>
+  <si>
+    <t>Jeseeta Appalasamy</t>
+  </si>
+  <si>
+    <t>Pannipa Phuangsaetsongsi</t>
+  </si>
+  <si>
+    <t>BACHELOR OF ARTS IN TEACHING</t>
+  </si>
+  <si>
+    <t>Airie Ginduk</t>
+  </si>
+  <si>
+    <t>Aye Nandar Ko</t>
+  </si>
+  <si>
+    <t>Cao Xinyi</t>
+  </si>
+  <si>
+    <t>Chen, Aiqiang</t>
+  </si>
+  <si>
+    <t>Elvica Lynn Wilson</t>
+  </si>
+  <si>
+    <t>Hong, Minghui</t>
+  </si>
+  <si>
+    <t>Ja Htoi Mai</t>
+  </si>
+  <si>
+    <t>Jesselyne  Ko Hui Lian</t>
+  </si>
+  <si>
+    <t>Kally Binti Sitim</t>
+  </si>
+  <si>
+    <t>Khun Kham Rhur</t>
+  </si>
+  <si>
+    <t>Kyal Sin Shin Thant</t>
+  </si>
+  <si>
+    <t>Liu Yuting</t>
+  </si>
+  <si>
+    <t>May Thazin Oo</t>
+  </si>
+  <si>
+    <t>Naw Htee Law Saw Paw</t>
+  </si>
+  <si>
+    <t>Naw Sara Hser Blut Htoo</t>
+  </si>
+  <si>
+    <t>Naw Ta Mu Lar Paw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nezi Mae Bacud Meringuez  </t>
+  </si>
+  <si>
+    <t>Pranee Wasuthanathee</t>
+  </si>
+  <si>
+    <t>Rebecca Thach</t>
+  </si>
+  <si>
+    <t>Saw Chit Oo</t>
+  </si>
+  <si>
+    <t>Saw Kyaw Lin Soe</t>
+  </si>
+  <si>
+    <t>Saw Plo Soe</t>
+  </si>
+  <si>
+    <t>Su Klay Moo</t>
+  </si>
+  <si>
+    <t>Su, Chunyu</t>
+  </si>
+  <si>
+    <t>Tha Th Yu Paw</t>
+  </si>
+  <si>
+    <t>Wang Bo</t>
+  </si>
+  <si>
+    <t>Wu, Xinyi</t>
+  </si>
+  <si>
+    <t>Yang YuYing</t>
+  </si>
+  <si>
+    <t>Yang, Deyi</t>
+  </si>
+  <si>
+    <t>Yoon Thiri</t>
+  </si>
+  <si>
+    <t>Zekiah KK Assan @ Artinih</t>
+  </si>
+  <si>
+    <t>Zhang, Jingru</t>
+  </si>
+  <si>
+    <t>Zhuang, Jiayin</t>
+  </si>
+  <si>
+    <t>BACHELOR OF BUSINESS ADMINISTRATION</t>
+  </si>
+  <si>
+    <t>Emphasis in Accounting</t>
+  </si>
+  <si>
+    <t>Enoch Chai Chuan Xun</t>
+  </si>
+  <si>
+    <t>Horng Phallavy</t>
+  </si>
+  <si>
+    <t>Jesson Lu Cueno Abragan</t>
+  </si>
+  <si>
+    <t>Khwanphon Rakkeereekamnoedsakun</t>
+  </si>
+  <si>
+    <t>Lorinda Sein</t>
+  </si>
+  <si>
+    <t>Naw Lar Bway</t>
+  </si>
+  <si>
+    <t>Sisasakhe Moyo</t>
+  </si>
+  <si>
+    <t>Yang, Deguang</t>
+  </si>
+  <si>
+    <t>Emphasis in Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayele Ines Sarah Ayivi-Togbassa </t>
+  </si>
+  <si>
+    <t>Chanikarn Ngamlord</t>
+  </si>
+  <si>
+    <t>Chen, Gong</t>
+  </si>
+  <si>
+    <t>Joseph Khamis Sabet Mehany</t>
+  </si>
+  <si>
+    <t>Sally Leong</t>
+  </si>
+  <si>
+    <t>Vo Truong Tuan</t>
+  </si>
+  <si>
+    <t>BACHELOR OF EDUCATION PROGRAM IN ELEMENTARY EDUCATION</t>
+  </si>
+  <si>
+    <t>Hla Maung Than</t>
+  </si>
+  <si>
+    <t>BACHELOR OF NURSING SCIENCE</t>
+  </si>
+  <si>
+    <t>Allyn Desiree Piseo Agustin</t>
+  </si>
+  <si>
+    <t>Earvin Tagala Noay</t>
+  </si>
+  <si>
+    <t>Ezekiel Michael Cometa Morley</t>
+  </si>
+  <si>
+    <t>Mung Thawn Khai</t>
+  </si>
+  <si>
+    <t>Natasha Victor</t>
+  </si>
+  <si>
+    <t>Panpailin Phimonaree</t>
+  </si>
+  <si>
+    <t>Praewnapa  Kamalaskomol</t>
+  </si>
+  <si>
+    <t>Seeda Lor</t>
+  </si>
+  <si>
+    <t>BACHELOR OF SCIENCE IN INFORMATION TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>Brandon Jay Willton Bendah</t>
+  </si>
+  <si>
+    <t>Musonda Kankomba</t>
+  </si>
+  <si>
+    <t>Winia Nawasirikhun</t>
+  </si>
+  <si>
+    <t>Nguyen Van Tien</t>
+  </si>
+  <si>
+    <t>Songnam Saraphai</t>
+  </si>
+  <si>
+    <t>Zhou Dawei</t>
+  </si>
+  <si>
+    <t>BACHELOR OF SCIENCE IN BIOSCIENCE</t>
+  </si>
+  <si>
+    <t>Emphasis in Biology</t>
+  </si>
+  <si>
+    <t>Nealler Afee Annc Aning</t>
+  </si>
+  <si>
+    <t>James Wong Yung Khai</t>
+  </si>
+  <si>
+    <t>Nyeleti Ruby Mawela</t>
+  </si>
+  <si>
+    <t>Priyanshi Anand</t>
+  </si>
+  <si>
+    <t>Marie Ange Fanta Issa Medere</t>
+  </si>
+  <si>
+    <t>Emphasis in Clinical Lab</t>
+  </si>
+  <si>
+    <t>Nethan Jeramy  Jeyaraman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emphasis in Community Public Health </t>
+  </si>
+  <si>
+    <t>Arora Abigail Ronald</t>
+  </si>
+  <si>
+    <t>Alrey Neal Hendriks</t>
+  </si>
+  <si>
+    <t>Saw Soe Hlaing</t>
+  </si>
+  <si>
+    <t>Saw Praising</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,13 +380,55 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF4472C4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -92,8 +443,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,10 +801,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B2B88B5-4638-4548-BEC4-699CC7D723DB}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A123"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.88671875" customWidth="1"/>
+    <col min="1" max="1" width="38.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -439,34 +812,588 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>2</v>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="2"/>
+    </row>
+    <row r="29" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" s="4"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" s="2"/>
+    </row>
+    <row r="68" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A80" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A83" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A84" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A85" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A86" s="2"/>
+    </row>
+    <row r="87" spans="1:1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A87" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A89" s="2"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A90" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A92" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99" s="4"/>
+    </row>
+    <row r="100" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A105" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A106" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A107" s="4"/>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A108" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A109" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A111" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A112" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A115" s="2"/>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A116" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A117" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A118" s="4"/>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A119" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A123" s="8" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>